<commit_message>
report4 for historical metrics and heatmap removed
</commit_message>
<xml_diff>
--- a/outputs/report/optimized_plan.xlsx
+++ b/outputs/report/optimized_plan.xlsx
@@ -9,7 +9,6 @@
     <sheet name="Optimization occupancy" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Overflows" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Transfers" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Heatmap" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -163,36 +162,6 @@
     </indexedColors>
   </colors>
 </styleSheet>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <oneCellAnchor>
-    <from>
-      <col>0</col>
-      <colOff>0</colOff>
-      <row>3</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="10668000" cy="10058400"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="1" name="Image 1" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -484,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K43"/>
+  <dimension ref="A1:L71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -543,6 +512,11 @@
           <t>type of transfer</t>
         </is>
       </c>
+      <c r="L1" s="3" t="inlineStr">
+        <is>
+          <t>run_timestamp</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -575,6 +549,10 @@
       <c r="H2" t="n">
         <v>0</v>
       </c>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -607,11 +585,19 @@
       <c r="H3" t="n">
         <v>0</v>
       </c>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>2026-02-24 19:41:15</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-02-23</t>
+          <t>2026-02-25</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -625,45 +611,53 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E4" t="n">
         <v>13</v>
       </c>
       <c r="F4" t="n">
-        <v>38.5</v>
+        <v>30.8</v>
       </c>
       <c r="G4" t="n">
         <v>0</v>
       </c>
       <c r="H4" t="n">
         <v>0</v>
+      </c>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>2026-02-25 10:24:02</t>
+        </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-02-24</t>
+          <t>2026-02-23</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>3D</t>
+          <t>3B</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>3D-PEDIATRIE</t>
+          <t>3B-MERE ENFANT</t>
         </is>
       </c>
       <c r="D5" t="n">
         <v>5</v>
       </c>
       <c r="E5" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="F5" t="n">
-        <v>55.6</v>
+        <v>38.5</v>
       </c>
       <c r="G5" t="n">
         <v>0</v>
@@ -671,43 +665,55 @@
       <c r="H5" t="n">
         <v>0</v>
       </c>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-02-23</t>
+          <t>2026-02-26</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>3D</t>
+          <t>3B</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>3D-PEDIATRIE</t>
+          <t>3B-MERE ENFANT</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E6" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="F6" t="n">
-        <v>77.8</v>
+        <v>46.2</v>
       </c>
       <c r="G6" t="n">
         <v>0</v>
       </c>
       <c r="H6" t="n">
         <v>0</v>
+      </c>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>2026-02-26 11:10:31</t>
+        </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-02-24</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -721,109 +727,133 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E7" t="n">
         <v>9</v>
       </c>
       <c r="F7" t="n">
-        <v>66.7</v>
+        <v>55.6</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
       </c>
       <c r="H7" t="n">
         <v>0</v>
+      </c>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>2026-02-24 19:41:15</t>
+        </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-02-23</t>
+          <t>2026-02-25</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>3DPEDOPSY</t>
+          <t>3D</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>3D PEDOPSYCHIATRIE</t>
+          <t>3D-PEDIATRIE</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E8" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="F8" t="n">
-        <v>25</v>
+        <v>66.7</v>
       </c>
       <c r="G8" t="n">
         <v>0</v>
       </c>
       <c r="H8" t="n">
         <v>0</v>
+      </c>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>2026-02-25 10:24:02</t>
+        </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-02-26</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>3DPEDOPSY</t>
+          <t>3D</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>3D PEDOPSYCHIATRIE</t>
+          <t>3D-PEDIATRIE</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="E9" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="F9" t="n">
-        <v>25</v>
+        <v>77.8</v>
       </c>
       <c r="G9" t="n">
         <v>0</v>
       </c>
       <c r="H9" t="n">
         <v>0</v>
+      </c>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>2026-02-26 11:10:31</t>
+        </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-02-24</t>
+          <t>2026-02-23</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>3DPEDOPSY</t>
+          <t>3D</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>3D PEDOPSYCHIATRIE</t>
+          <t>3D-PEDIATRIE</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="E10" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="F10" t="n">
-        <v>0</v>
+        <v>77.8</v>
       </c>
       <c r="G10" t="n">
         <v>0</v>
@@ -831,6 +861,10 @@
       <c r="H10" t="n">
         <v>0</v>
       </c>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -840,124 +874,148 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>3F</t>
+          <t>3D</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>3F-EVAL./READAPTATION/AVC</t>
+          <t>3D-PEDIATRIE</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>17</v>
+        <v>6</v>
       </c>
       <c r="E11" t="n">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="F11" t="n">
-        <v>100</v>
+        <v>66.7</v>
       </c>
       <c r="G11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H11" t="n">
         <v>0</v>
       </c>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-02-24</t>
+          <t>2026-02-26</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>3F</t>
+          <t>3DPEDOPSY</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>3F-EVAL./READAPTATION/AVC</t>
+          <t>3D PEDOPSYCHIATRIE</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="E12" t="n">
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="F12" t="n">
-        <v>100</v>
+        <v>25</v>
       </c>
       <c r="G12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H12" t="n">
         <v>0</v>
+      </c>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>2026-02-26 11:10:31</t>
+        </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-02-23</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>3F</t>
+          <t>3DPEDOPSY</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>3F-EVAL./READAPTATION/AVC</t>
+          <t>3D PEDOPSYCHIATRIE</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="E13" t="n">
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="F13" t="n">
-        <v>100</v>
+        <v>25</v>
       </c>
       <c r="G13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H13" t="n">
         <v>0</v>
       </c>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-02-25</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>3FSP</t>
+          <t>3DPEDOPSY</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>3FSP-SOINS PALLIATIFS</t>
+          <t>3D PEDOPSYCHIATRIE</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E14" t="n">
         <v>4</v>
       </c>
       <c r="F14" t="n">
-        <v>100</v>
+        <v>25</v>
       </c>
       <c r="G14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H14" t="n">
         <v>0</v>
+      </c>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>2026-02-25 10:24:02</t>
+        </is>
       </c>
     </row>
     <row r="15">
@@ -968,28 +1026,36 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>3FSP</t>
+          <t>3DPEDOPSY</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>3FSP-SOINS PALLIATIFS</t>
+          <t>3D PEDOPSYCHIATRIE</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="E15" t="n">
         <v>4</v>
       </c>
       <c r="F15" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="G15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H15" t="n">
         <v>0</v>
+      </c>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr"/>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>2026-02-24 19:41:15</t>
+        </is>
       </c>
     </row>
     <row r="16">
@@ -1000,60 +1066,72 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>3FSP</t>
+          <t>3DPEDOPSY</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>3FSP-SOINS PALLIATIFS</t>
+          <t>3D PEDOPSYCHIATRIE</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E16" t="n">
         <v>4</v>
       </c>
       <c r="F16" t="n">
-        <v>100</v>
+        <v>25</v>
       </c>
       <c r="G16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H16" t="n">
         <v>0</v>
       </c>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr"/>
+      <c r="L16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-02-23</t>
+          <t>2026-02-26</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>4A</t>
+          <t>3F</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>4A-CHIR.GENERALE/GYN-ONCO/URO</t>
+          <t>3F-EVAL./READAPTATION/AVC</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E17" t="n">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="F17" t="n">
-        <v>74.09999999999999</v>
+        <v>100</v>
       </c>
       <c r="G17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H17" t="n">
         <v>0</v>
+      </c>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr"/>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>2026-02-26 11:10:31</t>
+        </is>
       </c>
     </row>
     <row r="18">
@@ -1064,60 +1142,72 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>4A</t>
+          <t>3F</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>4A-CHIR.GENERALE/GYN-ONCO/URO</t>
+          <t>3F-EVAL./READAPTATION/AVC</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="E18" t="n">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="F18" t="n">
-        <v>88.90000000000001</v>
+        <v>100</v>
       </c>
       <c r="G18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H18" t="n">
         <v>0</v>
       </c>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
+      <c r="L18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-02-24</t>
+          <t>2026-02-25</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>4A</t>
+          <t>3F</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>4A-CHIR.GENERALE/GYN-ONCO/URO</t>
+          <t>3F-EVAL./READAPTATION/AVC</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="E19" t="n">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="F19" t="n">
-        <v>81.5</v>
+        <v>100</v>
       </c>
       <c r="G19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H19" t="n">
         <v>0</v>
+      </c>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr"/>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>2026-02-25 10:24:02</t>
+        </is>
       </c>
     </row>
     <row r="20">
@@ -1128,28 +1218,36 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>4B</t>
+          <t>3F</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>4B-PSYCHIATRIE</t>
+          <t>3F-EVAL./READAPTATION/AVC</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E20" t="n">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="F20" t="n">
-        <v>83.3</v>
+        <v>100</v>
       </c>
       <c r="G20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H20" t="n">
         <v>0</v>
+      </c>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr"/>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>2026-02-24 19:41:15</t>
+        </is>
       </c>
     </row>
     <row r="21">
@@ -1160,86 +1258,98 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>4B</t>
+          <t>3F</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>4B-PSYCHIATRIE</t>
+          <t>3F-EVAL./READAPTATION/AVC</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E21" t="n">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="F21" t="n">
-        <v>83.3</v>
+        <v>100</v>
       </c>
       <c r="G21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H21" t="n">
         <v>0</v>
       </c>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr"/>
+      <c r="L21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-02-26</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>4B</t>
+          <t>3FSP</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>4B-PSYCHIATRIE</t>
+          <t>3FSP-SOINS PALLIATIFS</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>22</v>
+        <v>4</v>
       </c>
       <c r="E22" t="n">
-        <v>24</v>
+        <v>4</v>
       </c>
       <c r="F22" t="n">
-        <v>91.7</v>
+        <v>100</v>
       </c>
       <c r="G22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H22" t="n">
         <v>0</v>
+      </c>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr"/>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>2026-02-26 11:10:31</t>
+        </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-02-25</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>4C</t>
+          <t>3FSP</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>4C-MED GEN/INTERNE/TELEMETRIE</t>
+          <t>3FSP-SOINS PALLIATIFS</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>29</v>
+        <v>4</v>
       </c>
       <c r="E23" t="n">
-        <v>30</v>
+        <v>4</v>
       </c>
       <c r="F23" t="n">
-        <v>96.7</v>
+        <v>100</v>
       </c>
       <c r="G23" t="n">
         <v>1</v>
@@ -1247,102 +1357,126 @@
       <c r="H23" t="n">
         <v>0</v>
       </c>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="inlineStr"/>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>2026-02-25 10:24:02</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-02-24</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>4C</t>
+          <t>3FSP</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>4C-MED GEN/INTERNE/TELEMETRIE</t>
+          <t>3FSP-SOINS PALLIATIFS</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>28</v>
+        <v>4</v>
       </c>
       <c r="E24" t="n">
-        <v>30</v>
+        <v>4</v>
       </c>
       <c r="F24" t="n">
-        <v>93.3</v>
+        <v>100</v>
       </c>
       <c r="G24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H24" t="n">
         <v>0</v>
       </c>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr"/>
+      <c r="K24" t="inlineStr"/>
+      <c r="L24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-02-23</t>
+          <t>2026-02-24</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>4C</t>
+          <t>3FSP</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>4C-MED GEN/INTERNE/TELEMETRIE</t>
+          <t>3FSP-SOINS PALLIATIFS</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>28</v>
+        <v>4</v>
       </c>
       <c r="E25" t="n">
-        <v>30</v>
+        <v>4</v>
       </c>
       <c r="F25" t="n">
-        <v>93.3</v>
+        <v>100</v>
       </c>
       <c r="G25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H25" t="n">
         <v>0</v>
+      </c>
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="inlineStr"/>
+      <c r="K25" t="inlineStr"/>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>2026-02-24 19:41:15</t>
+        </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-02-23</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>4D</t>
+          <t>3FSP</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>4D ONCOLOGIE</t>
+          <t>3FSP-SOINS PALLIATIFS</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>20</v>
+        <v>4</v>
       </c>
       <c r="E26" t="n">
-        <v>23</v>
+        <v>4</v>
       </c>
       <c r="F26" t="n">
-        <v>87</v>
+        <v>100</v>
       </c>
       <c r="G26" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H26" t="n">
         <v>0</v>
       </c>
+      <c r="I26" t="inlineStr"/>
+      <c r="J26" t="inlineStr"/>
+      <c r="K26" t="inlineStr"/>
+      <c r="L26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1352,22 +1486,22 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>4D</t>
+          <t>4A</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>4D ONCOLOGIE</t>
+          <t>4A-CHIR.GENERALE/GYN-ONCO/URO</t>
         </is>
       </c>
       <c r="D27" t="n">
         <v>20</v>
       </c>
       <c r="E27" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="F27" t="n">
-        <v>87</v>
+        <v>74.09999999999999</v>
       </c>
       <c r="G27" t="n">
         <v>0</v>
@@ -1375,31 +1509,35 @@
       <c r="H27" t="n">
         <v>0</v>
       </c>
+      <c r="I27" t="inlineStr"/>
+      <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr"/>
+      <c r="L27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-02-24</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>4D</t>
+          <t>4A</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>4D ONCOLOGIE</t>
+          <t>4A-CHIR.GENERALE/GYN-ONCO/URO</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="E28" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="F28" t="n">
-        <v>87</v>
+        <v>88.90000000000001</v>
       </c>
       <c r="G28" t="n">
         <v>0</v>
@@ -1407,6 +1545,10 @@
       <c r="H28" t="n">
         <v>0</v>
       </c>
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr"/>
+      <c r="K28" t="inlineStr"/>
+      <c r="L28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1416,195 +1558,196 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>4E</t>
+          <t>4A</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>4E-ORTHOPEDIE/ORL/PLASTIE</t>
+          <t>4A-CHIR.GENERALE/GYN-ONCO/URO</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="E29" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="F29" t="n">
-        <v>100</v>
+        <v>81.5</v>
       </c>
       <c r="G29" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H29" t="n">
         <v>0</v>
       </c>
-      <c r="I29" t="inlineStr">
-        <is>
-          <t>3D</t>
-        </is>
-      </c>
-      <c r="J29" t="n">
-        <v>1</v>
-      </c>
-      <c r="K29" t="inlineStr">
-        <is>
-          <t>backlog</t>
+      <c r="I29" t="inlineStr"/>
+      <c r="J29" t="inlineStr"/>
+      <c r="K29" t="inlineStr"/>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>2026-02-24 19:41:15</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-02-26</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>4E</t>
+          <t>4A</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>4E-ORTHOPEDIE/ORL/PLASTIE</t>
+          <t>4A-CHIR.GENERALE/GYN-ONCO/URO</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="E30" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="F30" t="n">
-        <v>100</v>
+        <v>81.5</v>
       </c>
       <c r="G30" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H30" t="n">
         <v>0</v>
       </c>
-      <c r="I30" t="inlineStr">
-        <is>
-          <t>SCHIR</t>
-        </is>
-      </c>
-      <c r="J30" t="n">
-        <v>1</v>
-      </c>
-      <c r="K30" t="inlineStr">
-        <is>
-          <t>backlog</t>
+      <c r="I30" t="inlineStr"/>
+      <c r="J30" t="inlineStr"/>
+      <c r="K30" t="inlineStr"/>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>2026-02-26 11:10:31</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-02-23</t>
+          <t>2026-02-25</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>4E</t>
+          <t>4A</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>4E-ORTHOPEDIE/ORL/PLASTIE</t>
+          <t>4A-CHIR.GENERALE/GYN-ONCO/URO</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="E31" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="F31" t="n">
-        <v>100</v>
+        <v>85.2</v>
       </c>
       <c r="G31" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H31" t="n">
         <v>0</v>
       </c>
-      <c r="I31" t="inlineStr">
-        <is>
-          <t>SCHIR</t>
-        </is>
-      </c>
-      <c r="J31" t="n">
-        <v>2</v>
-      </c>
-      <c r="K31" t="inlineStr">
-        <is>
-          <t>backlog</t>
+      <c r="I31" t="inlineStr"/>
+      <c r="J31" t="inlineStr"/>
+      <c r="K31" t="inlineStr"/>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>2026-02-25 10:24:02</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-02-25</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>4F</t>
+          <t>4B</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>4F-NEPHROLOGIE</t>
+          <t>4B-PSYCHIATRIE</t>
         </is>
       </c>
       <c r="D32" t="n">
         <v>19</v>
       </c>
       <c r="E32" t="n">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="F32" t="n">
-        <v>100</v>
+        <v>79.2</v>
       </c>
       <c r="G32" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H32" t="n">
         <v>0</v>
+      </c>
+      <c r="I32" t="inlineStr"/>
+      <c r="J32" t="inlineStr"/>
+      <c r="K32" t="inlineStr"/>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>2026-02-25 10:24:02</t>
+        </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-02-23</t>
+          <t>2026-02-26</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>4F</t>
+          <t>4B</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>4F-NEPHROLOGIE</t>
+          <t>4B-PSYCHIATRIE</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E33" t="n">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="F33" t="n">
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="G33" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H33" t="n">
         <v>0</v>
+      </c>
+      <c r="I33" t="inlineStr"/>
+      <c r="J33" t="inlineStr"/>
+      <c r="K33" t="inlineStr"/>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>2026-02-26 11:10:31</t>
+        </is>
       </c>
     </row>
     <row r="34">
@@ -1615,54 +1758,62 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>4F</t>
+          <t>4B</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>4F-NEPHROLOGIE</t>
+          <t>4B-PSYCHIATRIE</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E34" t="n">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="F34" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="G34" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H34" t="n">
         <v>0</v>
+      </c>
+      <c r="I34" t="inlineStr"/>
+      <c r="J34" t="inlineStr"/>
+      <c r="K34" t="inlineStr"/>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>2026-02-24 19:41:15</t>
+        </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-02-24</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>SCHIR</t>
+          <t>4B</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>SOINS INT MED CHIRURGICAUX</t>
+          <t>4B-PSYCHIATRIE</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="E35" t="n">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="F35" t="n">
-        <v>80</v>
+        <v>91.7</v>
       </c>
       <c r="G35" t="n">
         <v>0</v>
@@ -1670,31 +1821,35 @@
       <c r="H35" t="n">
         <v>0</v>
       </c>
+      <c r="I35" t="inlineStr"/>
+      <c r="J35" t="inlineStr"/>
+      <c r="K35" t="inlineStr"/>
+      <c r="L35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-02-23</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>SCHIR</t>
+          <t>4B</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>SOINS INT MED CHIRURGICAUX</t>
+          <t>4B-PSYCHIATRIE</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="E36" t="n">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="F36" t="n">
-        <v>90</v>
+        <v>83.3</v>
       </c>
       <c r="G36" t="n">
         <v>0</v>
@@ -1702,6 +1857,10 @@
       <c r="H36" t="n">
         <v>0</v>
       </c>
+      <c r="I36" t="inlineStr"/>
+      <c r="J36" t="inlineStr"/>
+      <c r="K36" t="inlineStr"/>
+      <c r="L36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1711,22 +1870,22 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>SCHIR</t>
+          <t>4C</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>SOINS INT MED CHIRURGICAUX</t>
+          <t>4C-MED GEN/INTERNE/TELEMETRIE</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>9</v>
+        <v>28</v>
       </c>
       <c r="E37" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="F37" t="n">
-        <v>90</v>
+        <v>93.3</v>
       </c>
       <c r="G37" t="n">
         <v>0</v>
@@ -1734,63 +1893,75 @@
       <c r="H37" t="n">
         <v>0</v>
       </c>
+      <c r="I37" t="inlineStr"/>
+      <c r="J37" t="inlineStr"/>
+      <c r="K37" t="inlineStr"/>
+      <c r="L37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-02-24</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>SCOR</t>
+          <t>4C</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>SOINS CORONARIENS</t>
+          <t>4C-MED GEN/INTERNE/TELEMETRIE</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>6</v>
+        <v>28</v>
       </c>
       <c r="E38" t="n">
-        <v>6</v>
+        <v>30</v>
       </c>
       <c r="F38" t="n">
-        <v>100</v>
+        <v>93.3</v>
       </c>
       <c r="G38" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H38" t="n">
         <v>0</v>
+      </c>
+      <c r="I38" t="inlineStr"/>
+      <c r="J38" t="inlineStr"/>
+      <c r="K38" t="inlineStr"/>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>2026-02-24 19:41:15</t>
+        </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-02-23</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>SCOR</t>
+          <t>4C</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>SOINS CORONARIENS</t>
+          <t>4C-MED GEN/INTERNE/TELEMETRIE</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>6</v>
+        <v>29</v>
       </c>
       <c r="E39" t="n">
-        <v>6</v>
+        <v>30</v>
       </c>
       <c r="F39" t="n">
-        <v>100</v>
+        <v>96.7</v>
       </c>
       <c r="G39" t="n">
         <v>1</v>
@@ -1798,95 +1969,115 @@
       <c r="H39" t="n">
         <v>0</v>
       </c>
+      <c r="I39" t="inlineStr"/>
+      <c r="J39" t="inlineStr"/>
+      <c r="K39" t="inlineStr"/>
+      <c r="L39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-02-24</t>
+          <t>2026-02-26</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>SCOR</t>
+          <t>4C</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>SOINS CORONARIENS</t>
+          <t>4C-MED GEN/INTERNE/TELEMETRIE</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>4</v>
+        <v>28</v>
       </c>
       <c r="E40" t="n">
-        <v>6</v>
+        <v>30</v>
       </c>
       <c r="F40" t="n">
-        <v>66.7</v>
+        <v>93.3</v>
       </c>
       <c r="G40" t="n">
         <v>0</v>
       </c>
       <c r="H40" t="n">
         <v>0</v>
+      </c>
+      <c r="I40" t="inlineStr"/>
+      <c r="J40" t="inlineStr"/>
+      <c r="K40" t="inlineStr"/>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>2026-02-26 11:10:31</t>
+        </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-02-25</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>SINTER</t>
+          <t>4C</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>SOINS INTERMEDIAIRES</t>
+          <t>4C-MED GEN/INTERNE/TELEMETRIE</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>7</v>
+        <v>30</v>
       </c>
       <c r="E41" t="n">
-        <v>8</v>
+        <v>30</v>
       </c>
       <c r="F41" t="n">
-        <v>87.5</v>
+        <v>100</v>
       </c>
       <c r="G41" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H41" t="n">
         <v>0</v>
+      </c>
+      <c r="I41" t="inlineStr"/>
+      <c r="J41" t="inlineStr"/>
+      <c r="K41" t="inlineStr"/>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>2026-02-25 10:24:02</t>
+        </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-02-23</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>SINTER</t>
+          <t>4D</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>SOINS INTERMEDIAIRES</t>
+          <t>4D ONCOLOGIE</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="E42" t="n">
-        <v>8</v>
+        <v>23</v>
       </c>
       <c r="F42" t="n">
-        <v>87.5</v>
+        <v>87</v>
       </c>
       <c r="G42" t="n">
         <v>0</v>
@@ -1894,6 +2085,10 @@
       <c r="H42" t="n">
         <v>0</v>
       </c>
+      <c r="I42" t="inlineStr"/>
+      <c r="J42" t="inlineStr"/>
+      <c r="K42" t="inlineStr"/>
+      <c r="L42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -1903,28 +2098,1162 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
+          <t>4D</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>4D ONCOLOGIE</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>20</v>
+      </c>
+      <c r="E43" t="n">
+        <v>23</v>
+      </c>
+      <c r="F43" t="n">
+        <v>87</v>
+      </c>
+      <c r="G43" t="n">
+        <v>0</v>
+      </c>
+      <c r="H43" t="n">
+        <v>0</v>
+      </c>
+      <c r="I43" t="inlineStr"/>
+      <c r="J43" t="inlineStr"/>
+      <c r="K43" t="inlineStr"/>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>2026-02-24 19:41:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-02-25</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>4D</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>4D ONCOLOGIE</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>19</v>
+      </c>
+      <c r="E44" t="n">
+        <v>23</v>
+      </c>
+      <c r="F44" t="n">
+        <v>82.59999999999999</v>
+      </c>
+      <c r="G44" t="n">
+        <v>0</v>
+      </c>
+      <c r="H44" t="n">
+        <v>0</v>
+      </c>
+      <c r="I44" t="inlineStr"/>
+      <c r="J44" t="inlineStr"/>
+      <c r="K44" t="inlineStr"/>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>2026-02-25 10:24:02</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-02-26</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>4D</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>4D ONCOLOGIE</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>21</v>
+      </c>
+      <c r="E45" t="n">
+        <v>23</v>
+      </c>
+      <c r="F45" t="n">
+        <v>91.3</v>
+      </c>
+      <c r="G45" t="n">
+        <v>0</v>
+      </c>
+      <c r="H45" t="n">
+        <v>0</v>
+      </c>
+      <c r="I45" t="inlineStr"/>
+      <c r="J45" t="inlineStr"/>
+      <c r="K45" t="inlineStr"/>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>2026-02-26 11:10:31</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-02-23</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>4D</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>4D ONCOLOGIE</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>20</v>
+      </c>
+      <c r="E46" t="n">
+        <v>23</v>
+      </c>
+      <c r="F46" t="n">
+        <v>87</v>
+      </c>
+      <c r="G46" t="n">
+        <v>0</v>
+      </c>
+      <c r="H46" t="n">
+        <v>0</v>
+      </c>
+      <c r="I46" t="inlineStr"/>
+      <c r="J46" t="inlineStr"/>
+      <c r="K46" t="inlineStr"/>
+      <c r="L46" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-02-25</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>4E</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>4E-ORTHOPEDIE/ORL/PLASTIE</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>25</v>
+      </c>
+      <c r="E47" t="n">
+        <v>25</v>
+      </c>
+      <c r="F47" t="n">
+        <v>100</v>
+      </c>
+      <c r="G47" t="n">
+        <v>2</v>
+      </c>
+      <c r="H47" t="n">
+        <v>0</v>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
           <t>SINTER</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr">
+      <c r="J47" t="n">
+        <v>1</v>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>backlog</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>2026-02-25 10:24:02</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2026-02-26</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>4E</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>4E-ORTHOPEDIE/ORL/PLASTIE</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>25</v>
+      </c>
+      <c r="E48" t="n">
+        <v>25</v>
+      </c>
+      <c r="F48" t="n">
+        <v>100</v>
+      </c>
+      <c r="G48" t="n">
+        <v>2</v>
+      </c>
+      <c r="H48" t="n">
+        <v>0</v>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>SCHIR</t>
+        </is>
+      </c>
+      <c r="J48" t="n">
+        <v>1</v>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>backlog</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>2026-02-26 11:10:31</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2026-02-24</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>4E</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>4E-ORTHOPEDIE/ORL/PLASTIE</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>25</v>
+      </c>
+      <c r="E49" t="n">
+        <v>25</v>
+      </c>
+      <c r="F49" t="n">
+        <v>100</v>
+      </c>
+      <c r="G49" t="n">
+        <v>2</v>
+      </c>
+      <c r="H49" t="n">
+        <v>0</v>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>3D</t>
+        </is>
+      </c>
+      <c r="J49" t="n">
+        <v>1</v>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>backlog</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>2026-02-24 19:41:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2026-02-23</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>4E</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>4E-ORTHOPEDIE/ORL/PLASTIE</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>25</v>
+      </c>
+      <c r="E50" t="n">
+        <v>25</v>
+      </c>
+      <c r="F50" t="n">
+        <v>100</v>
+      </c>
+      <c r="G50" t="n">
+        <v>2</v>
+      </c>
+      <c r="H50" t="n">
+        <v>0</v>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>SCHIR</t>
+        </is>
+      </c>
+      <c r="J50" t="n">
+        <v>2</v>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>backlog</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>4E</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>4E-ORTHOPEDIE/ORL/PLASTIE</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>25</v>
+      </c>
+      <c r="E51" t="n">
+        <v>25</v>
+      </c>
+      <c r="F51" t="n">
+        <v>100</v>
+      </c>
+      <c r="G51" t="n">
+        <v>2</v>
+      </c>
+      <c r="H51" t="n">
+        <v>0</v>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>SCHIR</t>
+        </is>
+      </c>
+      <c r="J51" t="n">
+        <v>1</v>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>backlog</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>4F</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>4F-NEPHROLOGIE</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>19</v>
+      </c>
+      <c r="E52" t="n">
+        <v>19</v>
+      </c>
+      <c r="F52" t="n">
+        <v>100</v>
+      </c>
+      <c r="G52" t="n">
+        <v>1</v>
+      </c>
+      <c r="H52" t="n">
+        <v>0</v>
+      </c>
+      <c r="I52" t="inlineStr"/>
+      <c r="J52" t="inlineStr"/>
+      <c r="K52" t="inlineStr"/>
+      <c r="L52" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2026-02-23</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>4F</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>4F-NEPHROLOGIE</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>19</v>
+      </c>
+      <c r="E53" t="n">
+        <v>19</v>
+      </c>
+      <c r="F53" t="n">
+        <v>100</v>
+      </c>
+      <c r="G53" t="n">
+        <v>1</v>
+      </c>
+      <c r="H53" t="n">
+        <v>0</v>
+      </c>
+      <c r="I53" t="inlineStr"/>
+      <c r="J53" t="inlineStr"/>
+      <c r="K53" t="inlineStr"/>
+      <c r="L53" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2026-02-26</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>4F</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>4F-NEPHROLOGIE</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>19</v>
+      </c>
+      <c r="E54" t="n">
+        <v>19</v>
+      </c>
+      <c r="F54" t="n">
+        <v>100</v>
+      </c>
+      <c r="G54" t="n">
+        <v>1</v>
+      </c>
+      <c r="H54" t="n">
+        <v>0</v>
+      </c>
+      <c r="I54" t="inlineStr"/>
+      <c r="J54" t="inlineStr"/>
+      <c r="K54" t="inlineStr"/>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>2026-02-26 11:10:31</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2026-02-25</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>4F</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>4F-NEPHROLOGIE</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>19</v>
+      </c>
+      <c r="E55" t="n">
+        <v>19</v>
+      </c>
+      <c r="F55" t="n">
+        <v>100</v>
+      </c>
+      <c r="G55" t="n">
+        <v>1</v>
+      </c>
+      <c r="H55" t="n">
+        <v>0</v>
+      </c>
+      <c r="I55" t="inlineStr"/>
+      <c r="J55" t="inlineStr"/>
+      <c r="K55" t="inlineStr"/>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>2026-02-25 10:24:02</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2026-02-24</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>4F</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>4F-NEPHROLOGIE</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>19</v>
+      </c>
+      <c r="E56" t="n">
+        <v>19</v>
+      </c>
+      <c r="F56" t="n">
+        <v>100</v>
+      </c>
+      <c r="G56" t="n">
+        <v>1</v>
+      </c>
+      <c r="H56" t="n">
+        <v>0</v>
+      </c>
+      <c r="I56" t="inlineStr"/>
+      <c r="J56" t="inlineStr"/>
+      <c r="K56" t="inlineStr"/>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>2026-02-24 19:41:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2026-02-23</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>SCHIR</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>SOINS INT MED CHIRURGICAUX</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>9</v>
+      </c>
+      <c r="E57" t="n">
+        <v>10</v>
+      </c>
+      <c r="F57" t="n">
+        <v>90</v>
+      </c>
+      <c r="G57" t="n">
+        <v>0</v>
+      </c>
+      <c r="H57" t="n">
+        <v>0</v>
+      </c>
+      <c r="I57" t="inlineStr"/>
+      <c r="J57" t="inlineStr"/>
+      <c r="K57" t="inlineStr"/>
+      <c r="L57" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2026-02-24</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>SCHIR</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>SOINS INT MED CHIRURGICAUX</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>8</v>
+      </c>
+      <c r="E58" t="n">
+        <v>10</v>
+      </c>
+      <c r="F58" t="n">
+        <v>80</v>
+      </c>
+      <c r="G58" t="n">
+        <v>0</v>
+      </c>
+      <c r="H58" t="n">
+        <v>0</v>
+      </c>
+      <c r="I58" t="inlineStr"/>
+      <c r="J58" t="inlineStr"/>
+      <c r="K58" t="inlineStr"/>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>2026-02-24 19:41:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2026-02-25</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>SCHIR</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>SOINS INT MED CHIRURGICAUX</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>8</v>
+      </c>
+      <c r="E59" t="n">
+        <v>10</v>
+      </c>
+      <c r="F59" t="n">
+        <v>80</v>
+      </c>
+      <c r="G59" t="n">
+        <v>0</v>
+      </c>
+      <c r="H59" t="n">
+        <v>0</v>
+      </c>
+      <c r="I59" t="inlineStr"/>
+      <c r="J59" t="inlineStr"/>
+      <c r="K59" t="inlineStr"/>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>2026-02-25 10:24:02</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2026-02-26</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>SCHIR</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>SOINS INT MED CHIRURGICAUX</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>7</v>
+      </c>
+      <c r="E60" t="n">
+        <v>10</v>
+      </c>
+      <c r="F60" t="n">
+        <v>70</v>
+      </c>
+      <c r="G60" t="n">
+        <v>0</v>
+      </c>
+      <c r="H60" t="n">
+        <v>0</v>
+      </c>
+      <c r="I60" t="inlineStr"/>
+      <c r="J60" t="inlineStr"/>
+      <c r="K60" t="inlineStr"/>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>2026-02-26 11:10:31</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>SCHIR</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>SOINS INT MED CHIRURGICAUX</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>9</v>
+      </c>
+      <c r="E61" t="n">
+        <v>10</v>
+      </c>
+      <c r="F61" t="n">
+        <v>90</v>
+      </c>
+      <c r="G61" t="n">
+        <v>0</v>
+      </c>
+      <c r="H61" t="n">
+        <v>0</v>
+      </c>
+      <c r="I61" t="inlineStr"/>
+      <c r="J61" t="inlineStr"/>
+      <c r="K61" t="inlineStr"/>
+      <c r="L61" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>2026-02-23</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>SCOR</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>SOINS CORONARIENS</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>6</v>
+      </c>
+      <c r="E62" t="n">
+        <v>6</v>
+      </c>
+      <c r="F62" t="n">
+        <v>100</v>
+      </c>
+      <c r="G62" t="n">
+        <v>1</v>
+      </c>
+      <c r="H62" t="n">
+        <v>0</v>
+      </c>
+      <c r="I62" t="inlineStr"/>
+      <c r="J62" t="inlineStr"/>
+      <c r="K62" t="inlineStr"/>
+      <c r="L62" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2026-02-25</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>SCOR</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>SOINS CORONARIENS</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>6</v>
+      </c>
+      <c r="E63" t="n">
+        <v>6</v>
+      </c>
+      <c r="F63" t="n">
+        <v>100</v>
+      </c>
+      <c r="G63" t="n">
+        <v>1</v>
+      </c>
+      <c r="H63" t="n">
+        <v>0</v>
+      </c>
+      <c r="I63" t="inlineStr"/>
+      <c r="J63" t="inlineStr"/>
+      <c r="K63" t="inlineStr"/>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>2026-02-25 10:24:02</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>2026-02-24</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>SCOR</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>SOINS CORONARIENS</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>4</v>
+      </c>
+      <c r="E64" t="n">
+        <v>6</v>
+      </c>
+      <c r="F64" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="G64" t="n">
+        <v>0</v>
+      </c>
+      <c r="H64" t="n">
+        <v>0</v>
+      </c>
+      <c r="I64" t="inlineStr"/>
+      <c r="J64" t="inlineStr"/>
+      <c r="K64" t="inlineStr"/>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>2026-02-24 19:41:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>2026-02-26</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>SCOR</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>SOINS CORONARIENS</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>5</v>
+      </c>
+      <c r="E65" t="n">
+        <v>6</v>
+      </c>
+      <c r="F65" t="n">
+        <v>83.3</v>
+      </c>
+      <c r="G65" t="n">
+        <v>0</v>
+      </c>
+      <c r="H65" t="n">
+        <v>0</v>
+      </c>
+      <c r="I65" t="inlineStr"/>
+      <c r="J65" t="inlineStr"/>
+      <c r="K65" t="inlineStr"/>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>2026-02-26 11:10:31</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>SCOR</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>SOINS CORONARIENS</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>6</v>
+      </c>
+      <c r="E66" t="n">
+        <v>6</v>
+      </c>
+      <c r="F66" t="n">
+        <v>100</v>
+      </c>
+      <c r="G66" t="n">
+        <v>1</v>
+      </c>
+      <c r="H66" t="n">
+        <v>0</v>
+      </c>
+      <c r="I66" t="inlineStr"/>
+      <c r="J66" t="inlineStr"/>
+      <c r="K66" t="inlineStr"/>
+      <c r="L66" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>2026-02-25</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>SINTER</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
         <is>
           <t>SOINS INTERMEDIAIRES</t>
         </is>
       </c>
-      <c r="D43" t="n">
+      <c r="D67" t="n">
+        <v>7</v>
+      </c>
+      <c r="E67" t="n">
+        <v>8</v>
+      </c>
+      <c r="F67" t="n">
+        <v>87.5</v>
+      </c>
+      <c r="G67" t="n">
+        <v>0</v>
+      </c>
+      <c r="H67" t="n">
+        <v>0</v>
+      </c>
+      <c r="I67" t="inlineStr"/>
+      <c r="J67" t="inlineStr"/>
+      <c r="K67" t="inlineStr"/>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>2026-02-25 10:24:02</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>2026-02-23</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>SINTER</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>SOINS INTERMEDIAIRES</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>7</v>
+      </c>
+      <c r="E68" t="n">
+        <v>8</v>
+      </c>
+      <c r="F68" t="n">
+        <v>87.5</v>
+      </c>
+      <c r="G68" t="n">
+        <v>0</v>
+      </c>
+      <c r="H68" t="n">
+        <v>0</v>
+      </c>
+      <c r="I68" t="inlineStr"/>
+      <c r="J68" t="inlineStr"/>
+      <c r="K68" t="inlineStr"/>
+      <c r="L68" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>SINTER</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>SOINS INTERMEDIAIRES</t>
+        </is>
+      </c>
+      <c r="D69" t="n">
+        <v>7</v>
+      </c>
+      <c r="E69" t="n">
+        <v>8</v>
+      </c>
+      <c r="F69" t="n">
+        <v>87.5</v>
+      </c>
+      <c r="G69" t="n">
+        <v>0</v>
+      </c>
+      <c r="H69" t="n">
+        <v>0</v>
+      </c>
+      <c r="I69" t="inlineStr"/>
+      <c r="J69" t="inlineStr"/>
+      <c r="K69" t="inlineStr"/>
+      <c r="L69" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>2026-02-24</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>SINTER</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>SOINS INTERMEDIAIRES</t>
+        </is>
+      </c>
+      <c r="D70" t="n">
         <v>6</v>
       </c>
-      <c r="E43" t="n">
+      <c r="E70" t="n">
         <v>8</v>
       </c>
-      <c r="F43" t="n">
+      <c r="F70" t="n">
         <v>75</v>
       </c>
-      <c r="G43" t="n">
-        <v>0</v>
-      </c>
-      <c r="H43" t="n">
-        <v>0</v>
+      <c r="G70" t="n">
+        <v>0</v>
+      </c>
+      <c r="H70" t="n">
+        <v>0</v>
+      </c>
+      <c r="I70" t="inlineStr"/>
+      <c r="J70" t="inlineStr"/>
+      <c r="K70" t="inlineStr"/>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>2026-02-24 19:41:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>2026-02-26</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>SINTER</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>SOINS INTERMEDIAIRES</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>7</v>
+      </c>
+      <c r="E71" t="n">
+        <v>8</v>
+      </c>
+      <c r="F71" t="n">
+        <v>87.5</v>
+      </c>
+      <c r="G71" t="n">
+        <v>0</v>
+      </c>
+      <c r="H71" t="n">
+        <v>0</v>
+      </c>
+      <c r="I71" t="inlineStr"/>
+      <c r="J71" t="inlineStr"/>
+      <c r="K71" t="inlineStr"/>
+      <c r="L71" t="inlineStr">
+        <is>
+          <t>2026-02-26 11:10:31</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -1938,7 +3267,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:D1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1955,6 +3284,11 @@
       <c r="C1" s="3" t="inlineStr">
         <is>
           <t>overflows number</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>run_timestamp</t>
         </is>
       </c>
     </row>
@@ -1969,7 +3303,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1998,6 +3332,11 @@
           <t>type (new transfer or backlog)</t>
         </is>
       </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>run_timestamp</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -2023,6 +3362,7 @@
           <t>backlog</t>
         </is>
       </c>
+      <c r="F2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2048,6 +3388,7 @@
           <t>backlog</t>
         </is>
       </c>
+      <c r="F3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2071,39 +3412,75 @@
       <c r="E4" t="inlineStr">
         <is>
           <t>backlog</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>2026-02-24 19:41:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-02-25</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>4E</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>SINTER</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>backlog</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>2026-02-25 10:24:02</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-02-26</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>4E</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>SCHIR</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>backlog</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>2026-02-26 11:10:31</t>
         </is>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:A2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="3" t="inlineStr">
-        <is>
-          <t>Optimized occupancy heatmap — 2026-02-20 to 2026-02-24</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Cell label shows: % and occ/beds (+overflow if any)</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
run_pipeline running on task scheduler
</commit_message>
<xml_diff>
--- a/outputs/report/optimized_plan.xlsx
+++ b/outputs/report/optimized_plan.xlsx
@@ -706,7 +706,7 @@
       <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr">
         <is>
-          <t>2026-02-26 11:10:31</t>
+          <t>2026-02-26 13:34:16</t>
         </is>
       </c>
     </row>
@@ -826,7 +826,7 @@
       <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr">
         <is>
-          <t>2026-02-26 11:10:31</t>
+          <t>2026-02-26 13:34:16</t>
         </is>
       </c>
     </row>
@@ -938,7 +938,7 @@
       <c r="K12" t="inlineStr"/>
       <c r="L12" t="inlineStr">
         <is>
-          <t>2026-02-26 11:10:31</t>
+          <t>2026-02-26 13:34:16</t>
         </is>
       </c>
     </row>
@@ -1130,7 +1130,7 @@
       <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr">
         <is>
-          <t>2026-02-26 11:10:31</t>
+          <t>2026-02-26 13:34:16</t>
         </is>
       </c>
     </row>
@@ -1322,7 +1322,7 @@
       <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr">
         <is>
-          <t>2026-02-26 11:10:31</t>
+          <t>2026-02-26 13:34:16</t>
         </is>
       </c>
     </row>
@@ -1626,7 +1626,7 @@
       <c r="K30" t="inlineStr"/>
       <c r="L30" t="inlineStr">
         <is>
-          <t>2026-02-26 11:10:31</t>
+          <t>2026-02-26 13:34:16</t>
         </is>
       </c>
     </row>
@@ -1746,7 +1746,7 @@
       <c r="K33" t="inlineStr"/>
       <c r="L33" t="inlineStr">
         <is>
-          <t>2026-02-26 11:10:31</t>
+          <t>2026-02-26 13:34:16</t>
         </is>
       </c>
     </row>
@@ -2010,7 +2010,7 @@
       <c r="K40" t="inlineStr"/>
       <c r="L40" t="inlineStr">
         <is>
-          <t>2026-02-26 11:10:31</t>
+          <t>2026-02-26 13:34:16</t>
         </is>
       </c>
     </row>
@@ -2206,7 +2206,7 @@
       <c r="K45" t="inlineStr"/>
       <c r="L45" t="inlineStr">
         <is>
-          <t>2026-02-26 11:10:31</t>
+          <t>2026-02-26 13:34:16</t>
         </is>
       </c>
     </row>
@@ -2342,7 +2342,7 @@
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>2026-02-26 11:10:31</t>
+          <t>2026-02-26 13:34:16</t>
         </is>
       </c>
     </row>
@@ -2596,7 +2596,7 @@
       <c r="K54" t="inlineStr"/>
       <c r="L54" t="inlineStr">
         <is>
-          <t>2026-02-26 11:10:31</t>
+          <t>2026-02-26 13:34:16</t>
         </is>
       </c>
     </row>
@@ -2832,7 +2832,7 @@
       <c r="K60" t="inlineStr"/>
       <c r="L60" t="inlineStr">
         <is>
-          <t>2026-02-26 11:10:31</t>
+          <t>2026-02-26 13:34:16</t>
         </is>
       </c>
     </row>
@@ -3024,7 +3024,7 @@
       <c r="K65" t="inlineStr"/>
       <c r="L65" t="inlineStr">
         <is>
-          <t>2026-02-26 11:10:31</t>
+          <t>2026-02-26 13:34:16</t>
         </is>
       </c>
     </row>
@@ -3252,7 +3252,7 @@
       <c r="K71" t="inlineStr"/>
       <c r="L71" t="inlineStr">
         <is>
-          <t>2026-02-26 11:10:31</t>
+          <t>2026-02-26 13:34:16</t>
         </is>
       </c>
     </row>
@@ -3476,7 +3476,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026-02-26 11:10:31</t>
+          <t>2026-02-26 13:34:16</t>
         </is>
       </c>
     </row>

</xml_diff>